<commit_message>
Add usage data for 22 Oct 2026 (11 logins); merge 1 late 21 Oct login
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/daily_snapshots/Daily Usage Snapshot - 21-10-2026.xlsx
+++ b/daily_snapshots/Daily Usage Snapshot - 21-10-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1356,6 +1356,53 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>user1792417475.1854</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>kranskopprimary@gmail.com</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rohan</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Maharaj</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Wednesday, 21 October 2026 at 19:39</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Kranskop Primary School</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Classroom</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Paying</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>